<commit_message>
Week 1: Part 7: Updated the Linux Practice Log
</commit_message>
<xml_diff>
--- a/Week_1/01. Linux Practice Log.xlsx
+++ b/Week_1/01. Linux Practice Log.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/raichu1231/Desktop/F9_Internship/01. Deliverables/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/raichu1231/Desktop/F9_Internship/01. Deliverables/Week_1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{785029ED-8459-8349-9BB6-1FF40C255C5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6939F30-A7E5-AD44-B82E-0EF714227B81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14680" yWindow="660" windowWidth="14720" windowHeight="17120" xr2:uid="{73F62D21-268A-4D44-9C04-F5D094355DAD}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17120" xr2:uid="{73F62D21-268A-4D44-9C04-F5D094355DAD}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="128">
   <si>
     <t>Category</t>
   </si>
@@ -399,6 +399,27 @@
   </si>
   <si>
     <t xml:space="preserve">Networking and Remote Acccess </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Outputs the user ID, group ID and group memberships for the current or specified user. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Outputs the user ID, group ID and group memberships for the root user. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Displays working directory </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prints full path to the current user's home directory </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Displays all files and directories in current working directory </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lists all visible files and folders inside the home directory </t>
+  </si>
+  <si>
+    <t>Moves the user into the F9_Internship folder</t>
   </si>
 </sst>
 </file>
@@ -482,10 +503,10 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -903,7 +924,9 @@
       <c r="C5" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="D5" s="6"/>
+      <c r="D5" s="6" t="s">
+        <v>121</v>
+      </c>
       <c r="E5" s="5" t="s">
         <v>17</v>
       </c>
@@ -918,7 +941,9 @@
       <c r="C6" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="D6" s="6"/>
+      <c r="D6" s="6" t="s">
+        <v>122</v>
+      </c>
       <c r="E6" s="5" t="s">
         <v>19</v>
       </c>
@@ -948,7 +973,9 @@
       <c r="C8" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="D8" s="6"/>
+      <c r="D8" s="6" t="s">
+        <v>123</v>
+      </c>
       <c r="E8" s="5" t="s">
         <v>22</v>
       </c>
@@ -963,12 +990,14 @@
       <c r="C9" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="D9" s="6"/>
+      <c r="D9" s="6" t="s">
+        <v>124</v>
+      </c>
       <c r="E9" s="5" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:15" ht="23" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:15" ht="46" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
         <v>5</v>
       </c>
@@ -978,7 +1007,9 @@
       <c r="C10" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="D10" s="6"/>
+      <c r="D10" s="6" t="s">
+        <v>125</v>
+      </c>
       <c r="E10" s="5" t="s">
         <v>27</v>
       </c>
@@ -1003,7 +1034,9 @@
       <c r="C11" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="D11" s="6"/>
+      <c r="D11" s="6" t="s">
+        <v>126</v>
+      </c>
       <c r="E11" s="5" t="s">
         <v>24</v>
       </c>
@@ -1028,7 +1061,9 @@
       <c r="C12" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="D12" s="6"/>
+      <c r="D12" s="6" t="s">
+        <v>127</v>
+      </c>
       <c r="E12" s="5" t="s">
         <v>29</v>
       </c>
@@ -1105,7 +1140,9 @@
       <c r="D16" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="E16" s="5"/>
+      <c r="E16" s="5" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="17" spans="1:5" ht="23" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
@@ -1137,7 +1174,9 @@
       <c r="D18" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="E18" s="5"/>
+      <c r="E18" s="5" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="19" spans="1:5" ht="23" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
@@ -1186,7 +1225,9 @@
       <c r="D21" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="E21" s="5"/>
+      <c r="E21" s="5" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="22" spans="1:5" ht="32" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
@@ -1201,7 +1242,9 @@
       <c r="D22" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="E22" s="5"/>
+      <c r="E22" s="5" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="23" spans="1:5" ht="48" x14ac:dyDescent="0.3">
       <c r="A23" s="4" t="s">
@@ -1216,7 +1259,9 @@
       <c r="D23" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="E23" s="5"/>
+      <c r="E23" s="5" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="24" spans="1:5" ht="46" x14ac:dyDescent="0.3">
       <c r="A24" s="4" t="s">
@@ -1231,7 +1276,9 @@
       <c r="D24" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="E24" s="5"/>
+      <c r="E24" s="5" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="25" spans="1:5" ht="46" x14ac:dyDescent="0.3">
       <c r="A25" s="4" t="s">
@@ -1246,7 +1293,9 @@
       <c r="D25" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="E25" s="5"/>
+      <c r="E25" s="5" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="26" spans="1:5" ht="46" x14ac:dyDescent="0.3">
       <c r="A26" s="4" t="s">
@@ -1261,7 +1310,9 @@
       <c r="D26" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="E26" s="5"/>
+      <c r="E26" s="5" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="27" spans="1:5" ht="46" x14ac:dyDescent="0.3">
       <c r="A27" s="4" t="s">
@@ -1276,7 +1327,9 @@
       <c r="D27" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="E27" s="5"/>
+      <c r="E27" s="5" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="28" spans="1:5" ht="46" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
@@ -1291,7 +1344,9 @@
       <c r="D28" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="E28" s="5"/>
+      <c r="E28" s="5" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="29" spans="1:5" ht="48" x14ac:dyDescent="0.3">
       <c r="A29" s="4" t="s">
@@ -1467,13 +1522,13 @@
       <c r="A39" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="B39" s="10" t="s">
+      <c r="B39" s="9" t="s">
         <v>120</v>
       </c>
-      <c r="C39" s="9" t="s">
+      <c r="C39" s="10" t="s">
         <v>87</v>
       </c>
-      <c r="D39" s="10" t="s">
+      <c r="D39" s="9" t="s">
         <v>88</v>
       </c>
       <c r="E39" s="5" t="s">
@@ -1482,144 +1537,144 @@
     </row>
     <row r="40" spans="1:5" ht="32" x14ac:dyDescent="0.3">
       <c r="A40" s="8"/>
-      <c r="B40" s="10"/>
-      <c r="C40" s="9"/>
-      <c r="D40" s="10"/>
+      <c r="B40" s="9"/>
+      <c r="C40" s="10"/>
+      <c r="D40" s="9"/>
       <c r="E40" s="5" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A41" s="8"/>
-      <c r="B41" s="10"/>
-      <c r="C41" s="9"/>
-      <c r="D41" s="10"/>
+      <c r="B41" s="9"/>
+      <c r="C41" s="10"/>
+      <c r="D41" s="9"/>
       <c r="E41" s="5" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="42" spans="1:5" ht="32" x14ac:dyDescent="0.3">
       <c r="A42" s="8"/>
-      <c r="B42" s="10"/>
-      <c r="C42" s="9"/>
-      <c r="D42" s="10"/>
+      <c r="B42" s="9"/>
+      <c r="C42" s="10"/>
+      <c r="D42" s="9"/>
       <c r="E42" s="5" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A43" s="8"/>
-      <c r="B43" s="10"/>
-      <c r="C43" s="9"/>
-      <c r="D43" s="10"/>
+      <c r="B43" s="9"/>
+      <c r="C43" s="10"/>
+      <c r="D43" s="9"/>
       <c r="E43" s="5" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="44" spans="1:5" ht="32" x14ac:dyDescent="0.3">
       <c r="A44" s="8"/>
-      <c r="B44" s="10"/>
-      <c r="C44" s="9"/>
-      <c r="D44" s="10"/>
+      <c r="B44" s="9"/>
+      <c r="C44" s="10"/>
+      <c r="D44" s="9"/>
       <c r="E44" s="5" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A45" s="8"/>
-      <c r="B45" s="10"/>
-      <c r="C45" s="9"/>
-      <c r="D45" s="10"/>
+      <c r="B45" s="9"/>
+      <c r="C45" s="10"/>
+      <c r="D45" s="9"/>
       <c r="E45" s="5" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A46" s="8"/>
-      <c r="B46" s="10"/>
-      <c r="C46" s="9"/>
-      <c r="D46" s="10"/>
+      <c r="B46" s="9"/>
+      <c r="C46" s="10"/>
+      <c r="D46" s="9"/>
       <c r="E46" s="5" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A47" s="8"/>
-      <c r="B47" s="10"/>
-      <c r="C47" s="9"/>
-      <c r="D47" s="10"/>
+      <c r="B47" s="9"/>
+      <c r="C47" s="10"/>
+      <c r="D47" s="9"/>
       <c r="E47" s="5" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A48" s="8"/>
-      <c r="B48" s="10"/>
-      <c r="C48" s="9"/>
-      <c r="D48" s="10"/>
+      <c r="B48" s="9"/>
+      <c r="C48" s="10"/>
+      <c r="D48" s="9"/>
       <c r="E48" s="5" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="49" spans="1:5" ht="32" x14ac:dyDescent="0.3">
       <c r="A49" s="8"/>
-      <c r="B49" s="10"/>
-      <c r="C49" s="9"/>
-      <c r="D49" s="10"/>
+      <c r="B49" s="9"/>
+      <c r="C49" s="10"/>
+      <c r="D49" s="9"/>
       <c r="E49" s="5" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A50" s="8"/>
-      <c r="B50" s="10"/>
-      <c r="C50" s="9"/>
-      <c r="D50" s="10"/>
+      <c r="B50" s="9"/>
+      <c r="C50" s="10"/>
+      <c r="D50" s="9"/>
       <c r="E50" s="5" t="s">
         <v>100</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A51" s="8"/>
-      <c r="B51" s="10"/>
-      <c r="C51" s="9"/>
-      <c r="D51" s="10"/>
+      <c r="B51" s="9"/>
+      <c r="C51" s="10"/>
+      <c r="D51" s="9"/>
       <c r="E51" s="5" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A52" s="8"/>
-      <c r="B52" s="10"/>
-      <c r="C52" s="9"/>
-      <c r="D52" s="10"/>
+      <c r="B52" s="9"/>
+      <c r="C52" s="10"/>
+      <c r="D52" s="9"/>
       <c r="E52" s="5" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A53" s="8"/>
-      <c r="B53" s="10"/>
-      <c r="C53" s="9"/>
-      <c r="D53" s="10"/>
+      <c r="B53" s="9"/>
+      <c r="C53" s="10"/>
+      <c r="D53" s="9"/>
       <c r="E53" s="5" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A54" s="8"/>
-      <c r="B54" s="10"/>
-      <c r="C54" s="9"/>
-      <c r="D54" s="10"/>
+      <c r="B54" s="9"/>
+      <c r="C54" s="10"/>
+      <c r="D54" s="9"/>
       <c r="E54" s="5" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A55" s="8"/>
-      <c r="B55" s="10"/>
-      <c r="C55" s="9"/>
-      <c r="D55" s="10"/>
+      <c r="B55" s="9"/>
+      <c r="C55" s="10"/>
+      <c r="D55" s="9"/>
       <c r="E55" s="5" t="s">
         <v>105</v>
       </c>

</xml_diff>